<commit_message>
pats 表补齐 DSM 6.2.4（DS918+/DS3617xs），供 2in1 6.2 版本线取 PAT
官方 7.x 升级 API 不含 6.2（RR 24.4.0 起已移除 6.2），上游 pats.xlsx 也没有 6.2 行，dsm_setup 对 req=6.2.4 会匹配不到而回退到该型号最新 7.x 并报「PAT 版本不匹配」。getpats 现在固定补两条官方 URL（build 25556，型号中的 '+' 编码为 %2B，sum 全 0 跳过校验），并重新生成 docs/pats.xlsx 与 docs/pats.json。

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pats.xlsx
+++ b/docs/pats.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D822"/>
+  <dimension ref="A1:D824"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18500,6 +18500,50 @@
         </is>
       </c>
     </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>DS918+</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>6.2.4-25556-0</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>https://global.synologydownload.com/download/DSM/release/6.2.4/25556/DSM_DS918%2B_25556.pat</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>00000000000000000000000000000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>DS3617xs</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>6.2.4-25556-0</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>https://global.synologydownload.com/download/DSM/release/6.2.4/25556/DSM_DS3617xs_25556.pat</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>00000000000000000000000000000000</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>